<commit_message>
Update example-report.xlsx to match hierarchical format
</commit_message>
<xml_diff>
--- a/example-report.xlsx
+++ b/example-report.xlsx
@@ -397,145 +397,279 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:C34"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Course Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Term</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Question</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Mean Score</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Responses</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Comment</v>
+        <v>Bruce D'Arcus</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>CS 101: Intro to Programming</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Fall 2024</v>
-      </c>
-      <c r="C2" t="str">
-        <v>The course material was clear and organized.</v>
-      </c>
-      <c r="D2" t="str">
-        <v>4.5</v>
-      </c>
-      <c r="E2" t="str">
-        <v>35</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Great class, really enjoyed the assignments.</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>CS 101: Intro to Programming</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Fall 2024</v>
-      </c>
-      <c r="C3" t="str">
-        <v>The instructor was well-prepared for class.</v>
-      </c>
-      <c r="D3" t="str">
-        <v>4.8</v>
-      </c>
-      <c r="E3" t="str">
-        <v>35</v>
+        <v>Term:202410 - 202510</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
         <v>CS 101: Intro to Programming</v>
       </c>
-      <c r="B4" t="str">
-        <v>Fall 2024</v>
-      </c>
       <c r="C4" t="str">
-        <v>Upon reflection, this instructor is an effective teacher.</v>
-      </c>
-      <c r="D4" t="str">
-        <v>4.7</v>
-      </c>
-      <c r="E4" t="str">
-        <v>35</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Best intro CS class I've taken!</v>
+        <v>202410</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>CS 101: Intro to Programming</v>
+        <v>The course material was clear and organized.</v>
       </c>
       <c r="B5" t="str">
-        <v>Fall 2024</v>
-      </c>
-      <c r="C5" t="str">
+        <v>Crs Mean</v>
+      </c>
+      <c r="C5">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="str">
+        <v>Dept Mean</v>
+      </c>
+      <c r="C6">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="str">
+        <v>School Mean</v>
+      </c>
+      <c r="C7">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="str">
+        <v>Univ Mean</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>The instructor presents content clearly and understandably</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Crs Mean</v>
+      </c>
+      <c r="C9">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="str">
+        <v>Dept Mean</v>
+      </c>
+      <c r="C10">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="str">
+        <v>School Mean</v>
+      </c>
+      <c r="C11">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="str">
+        <v>Univ Mean</v>
+      </c>
+      <c r="C12">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Upon reflection, this instructor is an effective teacher.</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Crs Mean</v>
+      </c>
+      <c r="C13">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="str">
+        <v>Dept Mean</v>
+      </c>
+      <c r="C14">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="str">
+        <v>School Mean</v>
+      </c>
+      <c r="C15">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="str">
+        <v>Univ Mean</v>
+      </c>
+      <c r="C16">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
         <v>On a scale of 1-10, how effective are the teaching methods of this faculty member?</v>
       </c>
-      <c r="D5" t="str">
+      <c r="B17" t="str">
+        <v>Crs Mean</v>
+      </c>
+      <c r="C17">
         <v>9.2</v>
       </c>
-      <c r="E5" t="str">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
+    </row>
+    <row r="18">
+      <c r="B18" t="str">
+        <v>Dept Mean</v>
+      </c>
+      <c r="C18">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="str">
+        <v>School Mean</v>
+      </c>
+      <c r="C19">
+        <v>8.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="str">
+        <v>Univ Mean</v>
+      </c>
+      <c r="C20">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="str">
+        <v>Total Enrollments</v>
+      </c>
+      <c r="C21">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="str">
+        <v>Response Rate</v>
+      </c>
+      <c r="C22">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
         <v>ENG 200: Advanced Literature</v>
       </c>
-      <c r="B6" t="str">
-        <v>Spring 2025</v>
-      </c>
-      <c r="C6" t="str">
+      <c r="C24" t="str">
+        <v>202510</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
         <v>The reading list was engaging and relevant.</v>
       </c>
-      <c r="D6" t="str">
+      <c r="B25" t="str">
+        <v>Crs Mean</v>
+      </c>
+      <c r="C25">
         <v>4.2</v>
       </c>
-      <c r="E6" t="str">
-        <v>20</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Some readings were a bit dense, but overall good.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>ENG 200: Advanced Literature</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Spring 2025</v>
-      </c>
-      <c r="C7" t="str">
+    </row>
+    <row r="26">
+      <c r="B26" t="str">
+        <v>Dept Mean</v>
+      </c>
+      <c r="C26">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="str">
+        <v>School Mean</v>
+      </c>
+      <c r="C27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="str">
+        <v>Univ Mean</v>
+      </c>
+      <c r="C28">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
         <v>Upon reflection, this instructor is an effective teacher.</v>
       </c>
-      <c r="D7" t="str">
+      <c r="B29" t="str">
+        <v>Crs Mean</v>
+      </c>
+      <c r="C29">
         <v>4.5</v>
       </c>
-      <c r="E7" t="str">
-        <v>20</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Passionate about the subject matter.</v>
+    </row>
+    <row r="30">
+      <c r="B30" t="str">
+        <v>Dept Mean</v>
+      </c>
+      <c r="C30">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="str">
+        <v>School Mean</v>
+      </c>
+      <c r="C31">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="str">
+        <v>Univ Mean</v>
+      </c>
+      <c r="C32">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="str">
+        <v>Total Enrollments</v>
+      </c>
+      <c r="C33">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="str">
+        <v>Response Rate</v>
+      </c>
+      <c r="C34">
+        <v>0.72</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C34"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>